<commit_message>
all user stories in issue format
</commit_message>
<xml_diff>
--- a/V3_UserStories_notes.xlsx
+++ b/V3_UserStories_notes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\9tesSemester\Software Engineering II\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\9tesSemester\Software Engineering II\ProjectMachiKoro\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DA209A-E326-4B56-889A-32FA0A647011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BF21B76-9E2B-497B-9A66-275BA3ABC536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{D819E763-2AAE-4DD4-93FD-6CBC8370491E}"/>
+    <workbookView xWindow="14925" yWindow="0" windowWidth="13980" windowHeight="15585" xr2:uid="{D819E763-2AAE-4DD4-93FD-6CBC8370491E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="792">
   <si>
     <t>Grüne und Violette Gebäude generieren nur im eigenen Zug Einkommen, Blau und Rot auch wenn eine adere Spieler Würfelt</t>
   </si>
@@ -2278,6 +2278,159 @@
   </si>
   <si>
     <t>Keep sorting fast and responsive</t>
+  </si>
+  <si>
+    <t>as a player I want different categories of cards and within cathegories cards triggered by different dice reutls - with differnet effects.</t>
+  </si>
+  <si>
+    <t>as a player I want my card effects to trigger in the right order; red first, then purple, then blue and green</t>
+  </si>
+  <si>
+    <t>As a player, I want card effects to trigger in the correct order so that the game rules are applied consistently.</t>
+  </si>
+  <si>
+    <t>Card effects resolve in the following order:
+1 Red cards
+2 Purple cards
+3 Blue cards &amp; Green cards</t>
+  </si>
+  <si>
+    <t>Effects within each category are resolved correctly (e.g. per player/order rules)</t>
+  </si>
+  <si>
+    <t>Order is consistent for all players</t>
+  </si>
+  <si>
+    <t>Final game state reflects correct resolution order</t>
+  </si>
+  <si>
+    <t>No effects are skipped or applied twice</t>
+  </si>
+  <si>
+    <t>Backend must enforce ordering logic</t>
+  </si>
+  <si>
+    <t>Important for fairness and rule accuracy</t>
+  </si>
+  <si>
+    <t>As a player, I want cards to be grouped into categories and activated by different dice results so that gameplay has variety and strategy.</t>
+  </si>
+  <si>
+    <t>Cards are categorized (e.g. red, blue, green, purple)</t>
+  </si>
+  <si>
+    <t>Each card has defined activation conditions (dice values or ranges)</t>
+  </si>
+  <si>
+    <t>Dice roll triggers matching cards correctly</t>
+  </si>
+  <si>
+    <t>Different cards produce different effects</t>
+  </si>
+  <si>
+    <t>Multiple matching cards activate correctly in one roll</t>
+  </si>
+  <si>
+    <t>Backend should handle all activation rules</t>
+  </si>
+  <si>
+    <t>As a player, I want to access a settings screen so that I can adjust game or app preferences.</t>
+  </si>
+  <si>
+    <t>A “Settings” button is accessible (e.g. main screen or menu)</t>
+  </si>
+  <si>
+    <t>Pressing the button opens a settings screen</t>
+  </si>
+  <si>
+    <t>Settings options are clearly displayed</t>
+  </si>
+  <si>
+    <t>Changes can be made and saved</t>
+  </si>
+  <si>
+    <t>Settings persist across app sessions (if applicable)</t>
+  </si>
+  <si>
+    <t>Define which settings are included (audio, visuals, gameplay, etc.)</t>
+  </si>
+  <si>
+    <t>As a player, I want to see coins move from their source to their destination so that I understand transactions during the game.</t>
+  </si>
+  <si>
+    <t>When coins are gained or lost, a visual animation is shown</t>
+  </si>
+  <si>
+    <t>Animation indicates source (bank or player) and destination</t>
+  </si>
+  <si>
+    <t>Coin count updates match the animation</t>
+  </si>
+  <si>
+    <t>Animation is visible to all relevant players</t>
+  </si>
+  <si>
+    <t>Animation does not block gameplay unnecessarily</t>
+  </si>
+  <si>
+    <t>Keep animations short and clear</t>
+  </si>
+  <si>
+    <t>As a player, I want the option to continue playing after a player wins so that extended gameplay modes are possible.</t>
+  </si>
+  <si>
+    <t>Lobby setting determines whether the game ends on first win</t>
+  </si>
+  <si>
+    <t>If enabled:
+Game continues after a player completes all landmarks</t>
+  </si>
+  <si>
+    <t>If disabled:
+Game ends immediately on win</t>
+  </si>
+  <si>
+    <t>Players are informed of the current rule setting</t>
+  </si>
+  <si>
+    <t>UI clearly indicates whether the game will continue or end</t>
+  </si>
+  <si>
+    <t>Requires lobby configuration support</t>
+  </si>
+  <si>
+    <t>Impacts win condition handling</t>
+  </si>
+  <si>
+    <t>As a player, I want to view all cards available in the game so that I can learn and plan strategies.</t>
+  </si>
+  <si>
+    <t>A button or menu option opens a card library</t>
+  </si>
+  <si>
+    <t>All available cards are displayed</t>
+  </si>
+  <si>
+    <t>Each card shows:
+Name
+Cost
+Effect
+Activation condition</t>
+  </si>
+  <si>
+    <t>Cards are organized (e.g. by category or cost)</t>
+  </si>
+  <si>
+    <t>View is accessible outside of active gameplay (and optionally during)</t>
+  </si>
+  <si>
+    <t>Useful for onboarding and strategy</t>
+  </si>
+  <si>
+    <t>Could reuse card UI components</t>
+  </si>
+  <si>
+    <t>optional</t>
   </si>
 </sst>
 </file>
@@ -2333,7 +2486,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2373,6 +2526,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2452,7 +2611,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2512,6 +2671,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -9468,7 +9630,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="49" spans="5:21" ht="60" x14ac:dyDescent="0.25">
+    <row r="49" spans="5:34" ht="60" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>164</v>
       </c>
@@ -9478,14 +9640,36 @@
       <c r="J49" s="23" t="s">
         <v>301</v>
       </c>
-      <c r="T49" s="25" t="s">
-        <v>284</v>
-      </c>
-      <c r="U49" s="25" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="50" spans="5:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="T49" s="29" t="s">
+        <v>745</v>
+      </c>
+      <c r="U49" s="29"/>
+      <c r="X49" t="s">
+        <v>746</v>
+      </c>
+      <c r="Z49" s="28" t="s">
+        <v>747</v>
+      </c>
+      <c r="AA49" t="s">
+        <v>748</v>
+      </c>
+      <c r="AB49" t="s">
+        <v>749</v>
+      </c>
+      <c r="AC49" t="s">
+        <v>750</v>
+      </c>
+      <c r="AD49" t="s">
+        <v>751</v>
+      </c>
+      <c r="AG49" t="s">
+        <v>752</v>
+      </c>
+      <c r="AH49" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="50" spans="5:34" ht="60" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>169</v>
       </c>
@@ -9495,14 +9679,33 @@
       <c r="J50" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="T50" s="25" t="s">
-        <v>277</v>
-      </c>
-      <c r="U50" s="25" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="51" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="T50" s="29" t="s">
+        <v>744</v>
+      </c>
+      <c r="U50" s="29"/>
+      <c r="X50" t="s">
+        <v>754</v>
+      </c>
+      <c r="Z50" t="s">
+        <v>755</v>
+      </c>
+      <c r="AA50" t="s">
+        <v>756</v>
+      </c>
+      <c r="AB50" t="s">
+        <v>757</v>
+      </c>
+      <c r="AC50" t="s">
+        <v>758</v>
+      </c>
+      <c r="AD50" t="s">
+        <v>759</v>
+      </c>
+      <c r="AG50" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="51" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>165</v>
       </c>
@@ -9513,13 +9716,13 @@
         <v>305</v>
       </c>
       <c r="T51" s="25" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="U51" s="25" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="52" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="52" spans="5:34" ht="60" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>166</v>
       </c>
@@ -9528,13 +9731,13 @@
       </c>
       <c r="J52" s="1"/>
       <c r="T52" s="25" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="U52" s="25" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="53" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="53" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>168</v>
       </c>
@@ -9544,12 +9747,14 @@
       <c r="J53" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="T53" s="26"/>
+      <c r="T53" s="25" t="s">
+        <v>278</v>
+      </c>
       <c r="U53" s="25" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="54" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="54" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>170</v>
       </c>
@@ -9558,13 +9763,13 @@
       </c>
       <c r="J54" s="1"/>
       <c r="T54" s="25" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="U54" s="25" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="55" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="55" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>172</v>
       </c>
@@ -9574,24 +9779,22 @@
       <c r="J55" s="15" t="s">
         <v>311</v>
       </c>
-      <c r="T55" s="25" t="s">
-        <v>288</v>
-      </c>
+      <c r="T55" s="26"/>
       <c r="U55" s="25" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="56" spans="5:21" ht="60" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="56" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
       <c r="T56" s="25" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="U56" s="25" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="57" spans="5:21" ht="60" x14ac:dyDescent="0.25">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="57" spans="5:34" ht="60" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>179</v>
       </c>
@@ -9601,24 +9804,27 @@
       <c r="J57" s="15" t="s">
         <v>313</v>
       </c>
-      <c r="T57" s="27" t="s">
-        <v>234</v>
-      </c>
-      <c r="U57" s="27" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="58" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="T57" s="25" t="s">
+        <v>288</v>
+      </c>
+      <c r="U57" s="25" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="58" spans="5:34" ht="60" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>180</v>
       </c>
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
-      <c r="U58" s="27" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="59" spans="5:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="T58" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="U58" s="25" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="59" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="E59" t="s">
         <v>181</v>
       </c>
@@ -9629,23 +9835,68 @@
         <v>315</v>
       </c>
       <c r="T59" s="27" t="s">
-        <v>314</v>
+        <v>234</v>
       </c>
       <c r="U59" s="27" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="60" spans="5:21" ht="30" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+      <c r="W59" t="s">
+        <v>791</v>
+      </c>
+      <c r="X59" t="s">
+        <v>761</v>
+      </c>
+      <c r="Z59" t="s">
+        <v>762</v>
+      </c>
+      <c r="AA59" t="s">
+        <v>763</v>
+      </c>
+      <c r="AB59" t="s">
+        <v>764</v>
+      </c>
+      <c r="AC59" t="s">
+        <v>765</v>
+      </c>
+      <c r="AD59" t="s">
+        <v>766</v>
+      </c>
+      <c r="AG59" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="60" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
-      <c r="T60" s="27" t="s">
-        <v>327</v>
-      </c>
       <c r="U60" s="27" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="61" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+        <v>295</v>
+      </c>
+      <c r="W60" t="s">
+        <v>791</v>
+      </c>
+      <c r="X60" t="s">
+        <v>768</v>
+      </c>
+      <c r="Z60" t="s">
+        <v>769</v>
+      </c>
+      <c r="AA60" t="s">
+        <v>770</v>
+      </c>
+      <c r="AB60" t="s">
+        <v>771</v>
+      </c>
+      <c r="AC60" t="s">
+        <v>772</v>
+      </c>
+      <c r="AD60" t="s">
+        <v>773</v>
+      </c>
+      <c r="AG60" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="61" spans="5:34" ht="60" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
         <v>206</v>
       </c>
@@ -9655,8 +9906,41 @@
       <c r="J61" s="23" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="62" spans="5:21" ht="75" x14ac:dyDescent="0.25">
+      <c r="T61" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="U61" s="27" t="s">
+        <v>315</v>
+      </c>
+      <c r="W61" t="s">
+        <v>791</v>
+      </c>
+      <c r="X61" t="s">
+        <v>775</v>
+      </c>
+      <c r="Z61" t="s">
+        <v>776</v>
+      </c>
+      <c r="AA61" s="28" t="s">
+        <v>777</v>
+      </c>
+      <c r="AB61" s="28" t="s">
+        <v>778</v>
+      </c>
+      <c r="AC61" t="s">
+        <v>779</v>
+      </c>
+      <c r="AD61" t="s">
+        <v>780</v>
+      </c>
+      <c r="AG61" t="s">
+        <v>781</v>
+      </c>
+      <c r="AH61" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="62" spans="5:34" ht="75" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
         <v>207</v>
       </c>
@@ -9666,8 +9950,41 @@
       <c r="J62" s="23" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="63" spans="5:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="T62" s="27" t="s">
+        <v>327</v>
+      </c>
+      <c r="U62" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="W62" t="s">
+        <v>791</v>
+      </c>
+      <c r="X62" t="s">
+        <v>783</v>
+      </c>
+      <c r="Z62" t="s">
+        <v>784</v>
+      </c>
+      <c r="AA62" t="s">
+        <v>785</v>
+      </c>
+      <c r="AB62" s="28" t="s">
+        <v>786</v>
+      </c>
+      <c r="AC62" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD62" t="s">
+        <v>788</v>
+      </c>
+      <c r="AG62" t="s">
+        <v>789</v>
+      </c>
+      <c r="AH62" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="63" spans="5:34" ht="45" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
         <v>208</v>
       </c>
@@ -9678,7 +9995,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="64" spans="5:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="5:34" x14ac:dyDescent="0.25">
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
     </row>

</xml_diff>